<commit_message>
grain cropping enterprise, improve enterprise build and excel error detection
</commit_message>
<xml_diff>
--- a/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
+++ b/Excel/Enterprises/Enterprise_PastureBeef_Template_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\Enterprises\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9256770-0F63-4E93-9105-C317254B0803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20E2BFF-C80D-446E-B0C0-C59FCC44575C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="510" windowWidth="27450" windowHeight="15630" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="-90" yWindow="90" windowWidth="28800" windowHeight="17085" firstSheet="3" activeTab="7" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -326,7 +326,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="321">
   <si>
     <t>Home</t>
   </si>
@@ -1141,30 +1141,15 @@
     <t>Over 90%</t>
   </si>
   <si>
-    <t>Liveweight grown</t>
-  </si>
-  <si>
     <t>Between 21% and 50%</t>
   </si>
   <si>
-    <t>Manure produced</t>
-  </si>
-  <si>
     <t>Regional-level data from a government or industry database/survey</t>
   </si>
   <si>
     <t>Between 51% and 90%</t>
   </si>
   <si>
-    <t>Manure sold</t>
-  </si>
-  <si>
-    <t>Percent income from liveweight sold</t>
-  </si>
-  <si>
-    <t>Percent income from manure sold</t>
-  </si>
-  <si>
     <t>Site</t>
   </si>
   <si>
@@ -1177,93 +1162,21 @@
     <t>Pasture Beef</t>
   </si>
   <si>
-    <t>Livestock production region</t>
-  </si>
-  <si>
-    <t>Cattle breed</t>
-  </si>
-  <si>
-    <t>Head count</t>
-  </si>
-  <si>
-    <t>Liveweight</t>
-  </si>
-  <si>
-    <t>Liveweight gain</t>
-  </si>
-  <si>
     <t>Less than 20%</t>
   </si>
   <si>
-    <t>Dry matter digestibility of diet</t>
-  </si>
-  <si>
     <t>Unknown</t>
   </si>
   <si>
-    <t>Crude protein in diet</t>
-  </si>
-  <si>
-    <t>Livestock access to water bodies</t>
-  </si>
-  <si>
-    <t>Calving timing</t>
-  </si>
-  <si>
-    <t>Calving rates</t>
-  </si>
-  <si>
-    <t>Livestock sales</t>
-  </si>
-  <si>
-    <t>Livestock purchases</t>
-  </si>
-  <si>
     <t>Pasture management</t>
   </si>
   <si>
-    <t>Pasture type</t>
-  </si>
-  <si>
-    <t>Area under pasture</t>
-  </si>
-  <si>
-    <t>Pasture yield</t>
-  </si>
-  <si>
     <t>State-level data from a government or industry database/survey</t>
   </si>
   <si>
-    <t>Area of pasture renewed or removed</t>
-  </si>
-  <si>
     <t>Fertiliser applications</t>
   </si>
   <si>
-    <t>Branded inorganic fertiliser applications</t>
-  </si>
-  <si>
-    <t>Custom inorganic fertiliser blend applications</t>
-  </si>
-  <si>
-    <t>Lime applications</t>
-  </si>
-  <si>
-    <t>Organic fertiliser applications</t>
-  </si>
-  <si>
-    <t>Fuel consumption</t>
-  </si>
-  <si>
-    <t>Electricity consumption</t>
-  </si>
-  <si>
-    <t>Inbound freight use</t>
-  </si>
-  <si>
-    <t>Outbound freight use</t>
-  </si>
-  <si>
     <t>This location with spatial partitioning</t>
   </si>
   <si>
@@ -1297,22 +1210,10 @@
     <t>Data type</t>
   </si>
   <si>
-    <t>Fuel purchases</t>
-  </si>
-  <si>
-    <t>Electricity generation</t>
-  </si>
-  <si>
     <t>Fuel and electricity</t>
   </si>
   <si>
-    <t>Farm input purchases</t>
-  </si>
-  <si>
     <t>Farm input purchases, freight and waste outputs</t>
-  </si>
-  <si>
-    <t>Solid waste generation and treatment</t>
   </si>
   <si>
     <t>Total data quality score</t>
@@ -12385,7 +12286,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="94" t="s">
-        <v>313</v>
+        <v>280</v>
       </c>
       <c r="D1" s="94"/>
       <c r="E1" s="94"/>
@@ -12421,7 +12322,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="80" t="s">
-        <v>330</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -13013,7 +12914,7 @@
     </row>
     <row r="28" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D28" s="92" t="s">
-        <v>326</v>
+        <v>293</v>
       </c>
       <c r="E28" s="93"/>
       <c r="F28" s="93"/>
@@ -13034,13 +12935,13 @@
     <row r="30" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D31" s="80" t="s">
-        <v>327</v>
+        <v>294</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D33" s="12" t="s">
-        <v>328</v>
+        <v>295</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>8</v>
@@ -13089,7 +12990,7 @@
     </row>
     <row r="35" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D35" s="92" t="s">
-        <v>329</v>
+        <v>296</v>
       </c>
       <c r="E35" s="93"/>
       <c r="F35" s="93"/>
@@ -13110,12 +13011,12 @@
     <row r="37" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D38" s="80" t="s">
-        <v>331</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D39" s="12" t="s">
-        <v>332</v>
+        <v>299</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>8</v>
@@ -13136,7 +13037,7 @@
     </row>
     <row r="40" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D40" s="1" t="s">
-        <v>333</v>
+        <v>300</v>
       </c>
       <c r="E40" s="1" t="e" cm="1">
         <f t="array" ref="E40">VEERG_15_1_1_1__1_EmissionsFromPurchasedLivestock_Result_Method1</f>
@@ -13163,7 +13064,7 @@
     </row>
     <row r="41" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D41" s="1" t="s">
-        <v>334</v>
+        <v>301</v>
       </c>
       <c r="E41" s="1" t="e" cm="1">
         <f t="array" ref="E41">VEERG_15_2_1_1__1_EmissionsFromPurchasedFeed_Result_Method1</f>
@@ -13190,7 +13091,7 @@
     </row>
     <row r="42" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D42" s="1" t="s">
-        <v>335</v>
+        <v>302</v>
       </c>
       <c r="E42" s="1" t="e" cm="1">
         <f t="array" ref="E42">VEERG_15_3_1_1__1_EmissionsFromPurchasedMineralSupplements_Result_Method1</f>
@@ -13217,7 +13118,7 @@
     </row>
     <row r="43" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D43" s="1" t="s">
-        <v>336</v>
+        <v>303</v>
       </c>
       <c r="E43" s="1" t="e" cm="1">
         <f t="array" ref="E43">VEERG_15_4_1_1__2_EmissionsFromPurchasedFertiliserComponentsVariation_Result_Method1</f>
@@ -13244,7 +13145,7 @@
     </row>
     <row r="44" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D44" s="1" t="s">
-        <v>337</v>
+        <v>304</v>
       </c>
       <c r="E44" s="1" t="e" cm="1">
         <f t="array" ref="E44">VEERG_15_5_1_1__1_EmissionsFromPurchasedAgrichemicals_Result_Method1</f>
@@ -13271,7 +13172,7 @@
     </row>
     <row r="45" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D45" s="1" t="s">
-        <v>338</v>
+        <v>305</v>
       </c>
       <c r="E45" s="1" t="e" cm="1">
         <f t="array" ref="E45">VEERG_15_6_1_1__1_EmissionsFromPurchasedLime_Result_Method1</f>
@@ -13298,7 +13199,7 @@
     </row>
     <row r="46" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D46" s="1" t="s">
-        <v>339</v>
+        <v>306</v>
       </c>
       <c r="E46" s="1" t="e" cm="1">
         <f t="array" ref="E46">VEERG_15_7_1_1__1_EmissionsFromPurchasedServices_Result_Method1</f>
@@ -13325,7 +13226,7 @@
     </row>
     <row r="47" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D47" s="1" t="s">
-        <v>340</v>
+        <v>307</v>
       </c>
       <c r="E47" s="1" t="e" cm="1">
         <f t="array" ref="E47">VEERG_15_10_1_1__1_OtherPurchasedGoodsAndServices_CleaningChemicals_Result_Method1</f>
@@ -13352,7 +13253,7 @@
     </row>
     <row r="48" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D48" s="1" t="s">
-        <v>341</v>
+        <v>308</v>
       </c>
       <c r="E48" s="1" t="e" cm="1">
         <f t="array" ref="E48">VEERG_15_10_1_1__1_OtherPurchasedGoodsAndServices_PharmacyChemicals_Result_Method1</f>
@@ -13379,7 +13280,7 @@
     </row>
     <row r="49" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D49" s="1" t="s">
-        <v>342</v>
+        <v>309</v>
       </c>
       <c r="E49" s="1" t="e" cm="1">
         <f t="array" ref="E49">VEERG_15_10_1_1__1_OtherPurchasedGoodsAndServices_Misc_Result_Method1</f>
@@ -13406,7 +13307,7 @@
     </row>
     <row r="50" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D50" s="1" t="s">
-        <v>343</v>
+        <v>310</v>
       </c>
       <c r="E50" s="1" t="e" cm="1">
         <f t="array" ref="E50">VEERG_15_10_1_1__1_OtherPurchasedGoodsAndServices_Uncategorised_Result_Method1</f>
@@ -13433,7 +13334,7 @@
     </row>
     <row r="51" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D51" s="1" t="s">
-        <v>344</v>
+        <v>311</v>
       </c>
       <c r="E51" s="1" t="e" cm="1">
         <f t="array" ref="E51">VEERG_15_11_1_1__1_TotalUpstreamEmissionsFromFuel_Result</f>
@@ -13488,7 +13389,7 @@
     </row>
     <row r="53" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D53" s="1" t="s">
-        <v>345</v>
+        <v>312</v>
       </c>
       <c r="E53" s="1" t="e" cm="1">
         <f t="array" ref="E53">VEERG_15_14_1_1__1_EmbeddedEmissionsFromUpstreamFreight_Incoming_Result_Method1</f>
@@ -13515,7 +13416,7 @@
     </row>
     <row r="54" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D54" s="1" t="s">
-        <v>346</v>
+        <v>313</v>
       </c>
       <c r="E54" s="1" t="e" cm="1">
         <f t="array" ref="E54">VEERG_10_1_1_1__1_EmissionsFromWasteManagement_Scope3_Result_Method1</f>
@@ -13542,7 +13443,7 @@
     </row>
     <row r="55" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D55" s="1" t="s">
-        <v>347</v>
+        <v>314</v>
       </c>
       <c r="E55" s="1" t="e" cm="1">
         <f t="array" ref="E55">VEERG_15_14_1_1__1_EmbeddedEmissionsFromUpstreamFreight_Outgoing_Result_Method1</f>
@@ -13569,7 +13470,7 @@
     </row>
     <row r="56" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D56" s="92" t="s">
-        <v>348</v>
+        <v>315</v>
       </c>
       <c r="E56" s="93"/>
       <c r="F56" s="93"/>
@@ -13597,7 +13498,7 @@
     <row r="60" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="61" spans="4:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D61" s="92" t="s">
-        <v>323</v>
+        <v>290</v>
       </c>
       <c r="E61" s="93">
         <f>SUM(Table_Input_Enterprise_PlantingRemovals[Removal allocated to this enterprise])</f>
@@ -13627,7 +13528,7 @@
     </row>
     <row r="67" spans="4:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D67" s="90" t="s">
-        <v>353</v>
+        <v>320</v>
       </c>
       <c r="E67" s="91" t="e">
         <f>Result_Enterprise_Scope1_Method1+Result_Enterprise_Scope2_Method1+Result_Enterprise_Scope3_Method1</f>
@@ -13638,12 +13539,12 @@
         <v>#NAME?</v>
       </c>
       <c r="G67" s="98" t="s">
-        <v>325</v>
+        <v>292</v>
       </c>
     </row>
     <row r="68" spans="4:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D68" s="90" t="s">
-        <v>324</v>
+        <v>291</v>
       </c>
       <c r="E68" s="91" t="e">
         <f>Result_Enterprise_Gross_Method1-Result_Enterprise_Removals</f>
@@ -13654,7 +13555,7 @@
         <v>#NAME?</v>
       </c>
       <c r="G68" s="98" t="s">
-        <v>325</v>
+        <v>292</v>
       </c>
     </row>
     <row r="69" spans="4:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13690,7 +13591,7 @@
   <sheetData>
     <row r="1" spans="3:18" s="94" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
       <c r="C1" s="94" t="s">
-        <v>312</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" spans="3:18" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -13730,7 +13631,7 @@
     </row>
     <row r="36" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D36" s="78" t="s">
-        <v>322</v>
+        <v>289</v>
       </c>
       <c r="E36" s="1" t="e">
         <f>Result_EmissionsForWholeProductionCycle_Method1</f>
@@ -13746,7 +13647,7 @@
     </row>
     <row r="37" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D37" s="78" t="s">
-        <v>314</v>
+        <v>281</v>
       </c>
       <c r="E37" s="1" t="e">
         <f>Result_EmissionsForWholeProductionCycle_Method1-Result_CarbonRemovalsFromPlantings</f>
@@ -13788,16 +13689,16 @@
         <v>132</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>349</v>
+        <v>316</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>350</v>
+        <v>317</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>351</v>
+        <v>318</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>352</v>
+        <v>319</v>
       </c>
       <c r="J43" s="12" t="s">
         <v>130</v>
@@ -13991,10 +13892,10 @@
         <v>132</v>
       </c>
       <c r="F51" s="12" t="s">
-        <v>349</v>
+        <v>316</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>350</v>
+        <v>317</v>
       </c>
       <c r="H51" s="12" t="s">
         <v>174</v>
@@ -14173,10 +14074,10 @@
         <v>132</v>
       </c>
       <c r="F59" s="12" t="s">
-        <v>349</v>
+        <v>316</v>
       </c>
       <c r="G59" s="12" t="s">
-        <v>350</v>
+        <v>317</v>
       </c>
       <c r="H59" s="12"/>
       <c r="I59" s="12"/>
@@ -15283,7 +15184,7 @@
     </row>
     <row r="37" spans="4:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D37" s="2" t="s">
-        <v>320</v>
+        <v>287</v>
       </c>
     </row>
     <row r="40" spans="4:7" ht="18.75" x14ac:dyDescent="0.25">
@@ -15294,16 +15195,16 @@
     </row>
     <row r="42" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D42" s="21" t="s">
-        <v>315</v>
+        <v>282</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>316</v>
+        <v>283</v>
       </c>
       <c r="F42" s="21" t="s">
-        <v>317</v>
+        <v>284</v>
       </c>
       <c r="G42" s="83" t="s">
-        <v>319</v>
+        <v>286</v>
       </c>
     </row>
     <row r="43" spans="4:7" x14ac:dyDescent="0.25">
@@ -15317,7 +15218,7 @@
     </row>
     <row r="47" spans="4:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D47" s="2" t="s">
-        <v>321</v>
+        <v>288</v>
       </c>
     </row>
     <row r="49" spans="4:7" ht="18.75" x14ac:dyDescent="0.25">
@@ -15334,7 +15235,7 @@
     </row>
     <row r="52" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D52" s="1" t="s">
-        <v>318</v>
+        <v>285</v>
       </c>
     </row>
     <row r="54" spans="4:7" x14ac:dyDescent="0.25">
@@ -15856,7 +15757,7 @@
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.25">
       <c r="D7" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E7" s="83" t="s">
         <v>247</v>
@@ -15878,14 +15779,15 @@
       </c>
     </row>
     <row r="8" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D8" s="1" t="s">
-        <v>23</v>
+      <c r="D8" s="1" t="str">
+        <f>"Liveweight sold"</f>
+        <v>Liveweight sold</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>250</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>294</v>
+        <v>265</v>
       </c>
       <c r="G8" s="14" t="s">
         <v>252</v>
@@ -15898,17 +15800,18 @@
       </c>
     </row>
     <row r="9" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D9" s="1" t="s">
-        <v>253</v>
+      <c r="D9" s="1" t="str">
+        <f>"Liveweight grown"</f>
+        <v>Liveweight grown</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>251</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H9" s="84"/>
       <c r="I9" s="84"/>
@@ -15918,17 +15821,18 @@
       </c>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="1" t="str">
+        <f>"Manure produced"</f>
+        <v>Manure produced</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>255</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>263</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>257</v>
       </c>
       <c r="H10" s="84"/>
       <c r="I10" s="84"/>
@@ -15938,17 +15842,18 @@
       </c>
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D11" s="1" t="s">
-        <v>258</v>
+      <c r="D11" s="1" t="str">
+        <f>"Manure sold"</f>
+        <v>Manure sold</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>296</v>
+        <v>267</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="H11" s="84"/>
       <c r="I11" s="84"/>
@@ -15958,17 +15863,18 @@
       </c>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D12" s="1" t="s">
-        <v>259</v>
+      <c r="D12" s="1" t="str">
+        <f>"Percent income from liveweight sold"</f>
+        <v>Percent income from liveweight sold</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>297</v>
+        <v>268</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>295</v>
+        <v>266</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="H12" s="84"/>
       <c r="I12" s="84"/>
@@ -15978,8 +15884,9 @@
       </c>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D13" s="1" t="s">
-        <v>260</v>
+      <c r="D13" s="1" t="str">
+        <f>"Percent income from manure sold"</f>
+        <v>Percent income from manure sold</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>250</v>
@@ -16005,12 +15912,12 @@
     </row>
     <row r="16" spans="3:13" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D16" s="2" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D18" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E18" s="83" t="s">
         <v>247</v>
@@ -16032,14 +15939,15 @@
       </c>
     </row>
     <row r="19" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D19" s="1" t="s">
-        <v>113</v>
+      <c r="D19" s="1" t="str">
+        <f>"Leaching zone"</f>
+        <v>Leaching zone</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>252</v>
@@ -16052,14 +15960,15 @@
       </c>
     </row>
     <row r="20" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D20" s="1" t="s">
-        <v>46</v>
+      <c r="D20" s="1" t="str">
+        <f>"Elevation"</f>
+        <v>Elevation</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>252</v>
@@ -16072,14 +15981,15 @@
       </c>
     </row>
     <row r="21" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D21" s="1" t="s">
-        <v>116</v>
+      <c r="D21" s="1" t="str">
+        <f>"Average temperature for reporting period"</f>
+        <v>Average temperature for reporting period</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G21" s="14" t="s">
         <v>252</v>
@@ -16092,8 +16002,9 @@
       </c>
     </row>
     <row r="22" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D22" s="1" t="s">
-        <v>118</v>
+      <c r="D22" s="1" t="str">
+        <f>"Total rainfall for reporting period"</f>
+        <v>Total rainfall for reporting period</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>250</v>
@@ -16112,14 +16023,15 @@
       </c>
     </row>
     <row r="23" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D23" s="1" t="s">
-        <v>120</v>
+      <c r="D23" s="1" t="str">
+        <f>"Potential evapotranspiration for reporting period"</f>
+        <v>Potential evapotranspiration for reporting period</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G23" s="14" t="s">
         <v>252</v>
@@ -16132,14 +16044,15 @@
       </c>
     </row>
     <row r="24" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D24" s="1" t="s">
-        <v>121</v>
+      <c r="D24" s="1" t="str">
+        <f>"Number of frost days for reporting period"</f>
+        <v>Number of frost days for reporting period</v>
       </c>
       <c r="E24" s="85" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="F24" s="85" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G24" s="85" t="s">
         <v>252</v>
@@ -16159,12 +16072,12 @@
     </row>
     <row r="27" spans="4:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D27" s="2" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D29" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E29" s="83" t="s">
         <v>247</v>
@@ -16186,14 +16099,15 @@
       </c>
     </row>
     <row r="30" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D30" s="1" t="s">
-        <v>265</v>
+      <c r="D30" s="1" t="str">
+        <f>"Livestock production region"</f>
+        <v>Livestock production region</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>250</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>252</v>
@@ -16206,8 +16120,9 @@
       </c>
     </row>
     <row r="31" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D31" s="1" t="s">
-        <v>266</v>
+      <c r="D31" s="1" t="str">
+        <f>"Cattle breed"</f>
+        <v>Cattle breed</v>
       </c>
       <c r="E31" s="14" t="s">
         <v>250</v>
@@ -16226,8 +16141,9 @@
       </c>
     </row>
     <row r="32" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D32" s="1" t="s">
-        <v>267</v>
+      <c r="D32" s="1" t="str">
+        <f>"Head count"</f>
+        <v>Head count</v>
       </c>
       <c r="E32" s="14" t="s">
         <v>250</v>
@@ -16236,7 +16152,7 @@
         <v>251</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H32" s="84"/>
       <c r="I32" s="84"/>
@@ -16246,8 +16162,9 @@
       </c>
     </row>
     <row r="33" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D33" s="1" t="s">
-        <v>268</v>
+      <c r="D33" s="1" t="str">
+        <f>"Liveweight"</f>
+        <v>Liveweight</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>250</v>
@@ -16256,7 +16173,7 @@
         <v>251</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H33" s="84"/>
       <c r="I33" s="84"/>
@@ -16266,8 +16183,9 @@
       </c>
     </row>
     <row r="34" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D34" s="1" t="s">
-        <v>269</v>
+      <c r="D34" s="1" t="str">
+        <f>"Liveweight gain"</f>
+        <v>Liveweight gain</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>250</v>
@@ -16276,7 +16194,7 @@
         <v>251</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="H34" s="84"/>
       <c r="I34" s="84"/>
@@ -16286,17 +16204,18 @@
       </c>
     </row>
     <row r="35" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D35" s="1" t="s">
-        <v>271</v>
+      <c r="D35" s="1" t="str">
+        <f>"Dry matter digestibility of diet"</f>
+        <v>Dry matter digestibility of diet</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>250</v>
       </c>
       <c r="F35" s="85" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G35" s="85" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="H35" s="84"/>
       <c r="I35" s="84"/>
@@ -16306,17 +16225,18 @@
       </c>
     </row>
     <row r="36" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D36" s="1" t="s">
-        <v>273</v>
+      <c r="D36" s="1" t="str">
+        <f>"Crude protein in diet"</f>
+        <v>Crude protein in diet</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>250</v>
       </c>
       <c r="F36" s="85" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G36" s="85" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="H36" s="84"/>
       <c r="I36" s="84"/>
@@ -16326,8 +16246,9 @@
       </c>
     </row>
     <row r="37" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D37" s="1" t="s">
-        <v>274</v>
+      <c r="D37" s="1" t="str">
+        <f>"Livestock access to water bodies"</f>
+        <v>Livestock access to water bodies</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>250</v>
@@ -16346,8 +16267,9 @@
       </c>
     </row>
     <row r="38" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D38" s="1" t="s">
-        <v>275</v>
+      <c r="D38" s="1" t="str">
+        <f>"Calving timing"</f>
+        <v>Calving timing</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>250</v>
@@ -16356,7 +16278,7 @@
         <v>251</v>
       </c>
       <c r="G38" s="85" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H38" s="84"/>
       <c r="I38" s="84"/>
@@ -16366,8 +16288,9 @@
       </c>
     </row>
     <row r="39" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D39" s="1" t="s">
-        <v>276</v>
+      <c r="D39" s="1" t="str">
+        <f>"Calving rates"</f>
+        <v>Calving rates</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>250</v>
@@ -16376,7 +16299,7 @@
         <v>251</v>
       </c>
       <c r="G39" s="85" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H39" s="84"/>
       <c r="I39" s="84"/>
@@ -16386,8 +16309,9 @@
       </c>
     </row>
     <row r="40" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D40" s="1" t="s">
-        <v>277</v>
+      <c r="D40" s="1" t="str">
+        <f>"Livestock sales"</f>
+        <v>Livestock sales</v>
       </c>
       <c r="E40" s="14" t="s">
         <v>250</v>
@@ -16406,8 +16330,9 @@
       </c>
     </row>
     <row r="41" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D41" s="1" t="s">
-        <v>278</v>
+      <c r="D41" s="1" t="str">
+        <f>"Livestock purchases"</f>
+        <v>Livestock purchases</v>
       </c>
       <c r="E41" s="14" t="s">
         <v>250</v>
@@ -16433,12 +16358,12 @@
     </row>
     <row r="44" spans="4:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D44" s="2" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
     </row>
     <row r="46" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D46" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E46" s="83" t="s">
         <v>247</v>
@@ -16460,8 +16385,9 @@
       </c>
     </row>
     <row r="47" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D47" s="1" t="s">
-        <v>280</v>
+      <c r="D47" s="1" t="str">
+        <f>"Pasture type"</f>
+        <v>Pasture type</v>
       </c>
       <c r="E47" s="14" t="s">
         <v>250</v>
@@ -16480,8 +16406,9 @@
       </c>
     </row>
     <row r="48" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D48" s="1" t="s">
-        <v>73</v>
+      <c r="D48" s="1" t="str">
+        <f>"Irrigation method"</f>
+        <v>Irrigation method</v>
       </c>
       <c r="E48" s="14" t="s">
         <v>250</v>
@@ -16500,8 +16427,9 @@
       </c>
     </row>
     <row r="49" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D49" s="1" t="s">
-        <v>281</v>
+      <c r="D49" s="1" t="str">
+        <f>"Area under pasture"</f>
+        <v>Area under pasture</v>
       </c>
       <c r="E49" s="14" t="s">
         <v>250</v>
@@ -16520,17 +16448,18 @@
       </c>
     </row>
     <row r="50" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D50" s="1" t="s">
-        <v>282</v>
+      <c r="D50" s="1" t="str">
+        <f>"Pasture yield"</f>
+        <v>Pasture yield</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>250</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="H50" s="84"/>
       <c r="I50" s="84"/>
@@ -16540,8 +16469,9 @@
       </c>
     </row>
     <row r="51" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D51" s="1" t="s">
-        <v>284</v>
+      <c r="D51" s="1" t="str">
+        <f>"Area of pasture renewed or removed"</f>
+        <v>Area of pasture renewed or removed</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>250</v>
@@ -16567,12 +16497,12 @@
     </row>
     <row r="54" spans="4:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D54" s="2" t="s">
-        <v>285</v>
+        <v>264</v>
       </c>
     </row>
     <row r="56" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D56" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E56" s="83" t="s">
         <v>247</v>
@@ -16594,8 +16524,9 @@
       </c>
     </row>
     <row r="57" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D57" s="1" t="s">
-        <v>286</v>
+      <c r="D57" s="1" t="str">
+        <f>"Branded inorganic fertiliser applications"</f>
+        <v>Branded inorganic fertiliser applications</v>
       </c>
       <c r="E57" s="14" t="s">
         <v>250</v>
@@ -16604,7 +16535,7 @@
         <v>251</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H57" s="84"/>
       <c r="I57" s="84"/>
@@ -16614,8 +16545,9 @@
       </c>
     </row>
     <row r="58" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D58" s="1" t="s">
-        <v>287</v>
+      <c r="D58" s="1" t="str">
+        <f>"Custom inorganic fertiliser blend applications"</f>
+        <v>Custom inorganic fertiliser blend applications</v>
       </c>
       <c r="E58" s="14" t="s">
         <v>250</v>
@@ -16634,8 +16566,9 @@
       </c>
     </row>
     <row r="59" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D59" s="1" t="s">
-        <v>288</v>
+      <c r="D59" s="1" t="str">
+        <f>"Lime applications"</f>
+        <v>Lime applications</v>
       </c>
       <c r="E59" s="14" t="s">
         <v>250</v>
@@ -16654,8 +16587,9 @@
       </c>
     </row>
     <row r="60" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D60" s="1" t="s">
-        <v>289</v>
+      <c r="D60" s="1" t="str">
+        <f>"Organic fertiliser applications"</f>
+        <v>Organic fertiliser applications</v>
       </c>
       <c r="E60" s="14" t="s">
         <v>250</v>
@@ -16681,12 +16615,12 @@
     </row>
     <row r="63" spans="4:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D63" s="2" t="s">
-        <v>307</v>
+        <v>276</v>
       </c>
     </row>
     <row r="65" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D65" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E65" s="83" t="s">
         <v>247</v>
@@ -16708,8 +16642,9 @@
       </c>
     </row>
     <row r="66" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D66" s="1" t="s">
-        <v>305</v>
+      <c r="D66" s="1" t="str">
+        <f>"Fuel purchases"</f>
+        <v>Fuel purchases</v>
       </c>
       <c r="E66" s="14" t="s">
         <v>250</v>
@@ -16718,7 +16653,7 @@
         <v>251</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H66" s="84"/>
       <c r="I66" s="84"/>
@@ -16728,8 +16663,9 @@
       </c>
     </row>
     <row r="67" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D67" s="1" t="s">
-        <v>290</v>
+      <c r="D67" s="1" t="str">
+        <f>"Fuel consumption"</f>
+        <v>Fuel consumption</v>
       </c>
       <c r="E67" s="14" t="s">
         <v>250</v>
@@ -16748,8 +16684,9 @@
       </c>
     </row>
     <row r="68" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D68" s="1" t="s">
-        <v>291</v>
+      <c r="D68" s="1" t="str">
+        <f>"Electricity consumption"</f>
+        <v>Electricity consumption</v>
       </c>
       <c r="E68" s="14" t="s">
         <v>250</v>
@@ -16768,8 +16705,9 @@
       </c>
     </row>
     <row r="69" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D69" s="1" t="s">
-        <v>306</v>
+      <c r="D69" s="1" t="str">
+        <f>"Electricity generation"</f>
+        <v>Electricity generation</v>
       </c>
       <c r="E69" s="14" t="s">
         <v>250</v>
@@ -16795,12 +16733,12 @@
     </row>
     <row r="73" spans="4:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D73" s="2" t="s">
-        <v>309</v>
+        <v>277</v>
       </c>
     </row>
     <row r="75" spans="4:10" x14ac:dyDescent="0.25">
       <c r="D75" s="83" t="s">
-        <v>304</v>
+        <v>275</v>
       </c>
       <c r="E75" s="83" t="s">
         <v>247</v>
@@ -16822,8 +16760,9 @@
       </c>
     </row>
     <row r="76" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D76" s="1" t="s">
-        <v>308</v>
+      <c r="D76" s="1" t="str">
+        <f>"Farm input purchases"</f>
+        <v>Farm input purchases</v>
       </c>
       <c r="E76" s="14" t="s">
         <v>250</v>
@@ -16832,7 +16771,7 @@
         <v>251</v>
       </c>
       <c r="G76" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H76" s="84"/>
       <c r="I76" s="84"/>
@@ -16842,8 +16781,9 @@
       </c>
     </row>
     <row r="77" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D77" s="1" t="s">
-        <v>292</v>
+      <c r="D77" s="1" t="str">
+        <f>"Inbound freight use"</f>
+        <v>Inbound freight use</v>
       </c>
       <c r="E77" s="14" t="s">
         <v>250</v>
@@ -16862,8 +16802,9 @@
       </c>
     </row>
     <row r="78" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D78" s="1" t="s">
-        <v>293</v>
+      <c r="D78" s="1" t="str">
+        <f>"Outbound freight use"</f>
+        <v>Outbound freight use</v>
       </c>
       <c r="E78" s="14" t="s">
         <v>250</v>
@@ -16882,8 +16823,9 @@
       </c>
     </row>
     <row r="79" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D79" s="1" t="s">
-        <v>310</v>
+      <c r="D79" s="1" t="str">
+        <f>"Solid waste generation and treatment"</f>
+        <v>Solid waste generation and treatment</v>
       </c>
       <c r="E79" s="14" t="s">
         <v>250</v>
@@ -16909,7 +16851,7 @@
     </row>
     <row r="83" spans="4:10" ht="20.25" x14ac:dyDescent="0.25">
       <c r="D83" s="92" t="s">
-        <v>311</v>
+        <v>278</v>
       </c>
       <c r="E83" s="93" t="str">
         <f>(J15+J26+J43+J53+J62+J71+J81)&amp;" out of "&amp;((COUNT(Table_Input_DataQuality_Enterprise[Score])*15)+(COUNT(Table_Input_DataQuality_Site[Score])*15)+(COUNT(Table_Input_DataQuality_PastureBeef[Score])*15)+(COUNT(Table_Input_DataQuality_PastureManagement[Score])*15)+(COUNT(Table_Input_DataQuality_FertiliserApplications[Score])*15)+(COUNT(Table_Input_DataQuality_FuelElectricity[Score])*15)+(COUNT(Table_Input_DataQuality_FarmInputsFreightWaste[Score])*15))</f>
@@ -21075,7 +21017,7 @@
     </row>
     <row r="265" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D265" s="21" t="s">
-        <v>298</v>
+        <v>269</v>
       </c>
       <c r="E265" s="21" t="s">
         <v>204</v>
@@ -21107,7 +21049,7 @@
     </row>
     <row r="267" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D267" s="21" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="E267" s="21" t="s">
         <v>208</v>
@@ -21123,7 +21065,7 @@
     </row>
     <row r="268" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D268" s="21" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="E268" s="21" t="s">
         <v>209</v>
@@ -21139,7 +21081,7 @@
     </row>
     <row r="269" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D269" s="21" t="s">
-        <v>296</v>
+        <v>267</v>
       </c>
       <c r="E269" s="21" t="s">
         <v>211</v>
@@ -21155,7 +21097,7 @@
     </row>
     <row r="270" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D270" s="21" t="s">
-        <v>297</v>
+        <v>268</v>
       </c>
       <c r="E270" s="21" t="s">
         <v>213</v>
@@ -21176,7 +21118,7 @@
     </row>
     <row r="274" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D274" s="21" t="s">
-        <v>298</v>
+        <v>269</v>
       </c>
       <c r="E274" s="21" t="s">
         <v>204</v>
@@ -21192,7 +21134,7 @@
     </row>
     <row r="275" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D275" s="21" t="s">
-        <v>294</v>
+        <v>265</v>
       </c>
       <c r="E275" s="21" t="s">
         <v>216</v>
@@ -21224,7 +21166,7 @@
     </row>
     <row r="277" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D277" s="21" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E277" s="21" t="s">
         <v>219</v>
@@ -21240,7 +21182,7 @@
     </row>
     <row r="278" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D278" s="21" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="E278" s="21" t="s">
         <v>221</v>
@@ -21256,7 +21198,7 @@
     </row>
     <row r="279" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D279" s="21" t="s">
-        <v>295</v>
+        <v>266</v>
       </c>
       <c r="E279" s="21" t="s">
         <v>223</v>
@@ -21277,7 +21219,7 @@
     </row>
     <row r="283" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D283" s="21" t="s">
-        <v>298</v>
+        <v>269</v>
       </c>
       <c r="E283" s="21" t="s">
         <v>204</v>
@@ -21309,7 +21251,7 @@
     </row>
     <row r="285" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D285" s="21" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E285" s="21" t="s">
         <v>228</v>
@@ -21325,7 +21267,7 @@
     </row>
     <row r="286" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D286" s="21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E286" s="21" t="s">
         <v>230</v>
@@ -21341,7 +21283,7 @@
     </row>
     <row r="287" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D287" s="21" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="E287" s="21" t="s">
         <v>231</v>
@@ -21357,7 +21299,7 @@
     </row>
     <row r="288" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D288" s="21" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="E288" s="21" t="s">
         <v>233</v>
@@ -21378,7 +21320,7 @@
     </row>
     <row r="292" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D292" s="21" t="s">
-        <v>298</v>
+        <v>269</v>
       </c>
       <c r="E292" s="21" t="s">
         <v>204</v>
@@ -21394,7 +21336,7 @@
     </row>
     <row r="293" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D293" s="21" t="s">
-        <v>299</v>
+        <v>270</v>
       </c>
       <c r="E293" s="21" t="s">
         <v>236</v>
@@ -21410,7 +21352,7 @@
     </row>
     <row r="294" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D294" s="21" t="s">
-        <v>300</v>
+        <v>271</v>
       </c>
       <c r="E294" s="21" t="s">
         <v>238</v>
@@ -21426,7 +21368,7 @@
     </row>
     <row r="295" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D295" s="21" t="s">
-        <v>301</v>
+        <v>272</v>
       </c>
       <c r="E295" s="21" t="s">
         <v>240</v>
@@ -21442,7 +21384,7 @@
     </row>
     <row r="296" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D296" s="21" t="s">
-        <v>302</v>
+        <v>273</v>
       </c>
       <c r="E296" s="21" t="s">
         <v>242</v>
@@ -21458,7 +21400,7 @@
     </row>
     <row r="297" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D297" s="21" t="s">
-        <v>303</v>
+        <v>274</v>
       </c>
       <c r="E297" s="21" t="s">
         <v>244</v>
@@ -21502,6 +21444,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA0ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -21696,20 +21642,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA0ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -21720,7 +21653,24 @@
 </p:properties>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21739,23 +21689,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -21764,4 +21698,12 @@
     <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>